<commit_message>
a lo grande amb l'html
</commit_message>
<xml_diff>
--- a/data/sankey/sankey_nodes-ste.xlsx
+++ b/data/sankey/sankey_nodes-ste.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\vapor\data\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\sankey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00062D96-E5F2-4FF8-B8DC-CAF64BD8B6A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6641CBD-49CE-4C8E-9E10-D7BCD92E6898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -597,7 +597,7 @@
         <v>3.3</v>
       </c>
       <c r="I5" s="9">
-        <f t="shared" ref="I4:I14" si="1">PI()*(((G5-2*H5)*10^-3)^2)/4</f>
+        <f t="shared" ref="I5:I14" si="1">PI()*(((G5-2*H5)*10^-3)^2)/4</f>
         <v>1.4186929768786934E-2</v>
       </c>
       <c r="J5" s="3">

</xml_diff>

<commit_message>
Mapa en html en lloc de pyqt
</commit_message>
<xml_diff>
--- a/data/sankey/sankey_nodes-ste.xlsx
+++ b/data/sankey/sankey_nodes-ste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\sankey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9607397B-6516-403E-8F9E-30170CDDCA65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB4A65B-AA89-4CEF-8E03-75797E7EF4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="44">
   <si>
     <t>source</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>rgba(255,0,255, 0.8)</t>
+  </si>
+  <si>
+    <t>rgba(0,255,0,0.4)</t>
   </si>
 </sst>
 </file>
@@ -522,7 +525,7 @@
         <v>1.418693E-2</v>
       </c>
       <c r="H4" s="6">
-        <v>2.2999999999999998</v>
+        <v>2.5</v>
       </c>
       <c r="I4" s="5">
         <v>3.2629937999999997E-2</v>
@@ -555,7 +558,7 @@
         <v>4.53646E-3</v>
       </c>
       <c r="H5" s="6">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I5" s="5">
         <v>0</v>
@@ -759,7 +762,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -778,7 +781,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
@@ -987,7 +990,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5">

</xml_diff>